<commit_message>
feat: Update test cases
</commit_message>
<xml_diff>
--- a/docs/TestCases_TaoDonBanHang.xlsx
+++ b/docs/TestCases_TaoDonBanHang.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\DATN-automation-test\DATN_DangThiCamTu_v2\DATN_DangThiCamTu\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D7D54BAD-408B-4826-A388-672DEAE10BCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94BD3380-315D-4898-ADF5-897C647C6C15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,6 @@
     <sheet name="TestCases_TaoDonBanHang" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
-  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
@@ -59,13 +58,7 @@
     <t>A. KÍCH HOẠT LỆNH TẠO ĐƠN</t>
   </si>
   <si>
-    <t>CD_01</t>
-  </si>
-  <si>
     <t>Kích hoạt lệnh</t>
-  </si>
-  <si>
-    <t>TC_CD_01</t>
   </si>
   <si>
     <t>Functional</t>
@@ -89,9 +82,6 @@
 Tổng tiền = 65k, Tổng VAT = 5.85k, KH phải trả = 60.85k</t>
   </si>
   <si>
-    <t>TC_CD_02</t>
-  </si>
-  <si>
     <t>Tạo đơn bán hàng thành công bằng phím tắt (F9)</t>
   </si>
   <si>
@@ -102,21 +92,12 @@
 2. Quan sát</t>
   </si>
   <si>
-    <t>Cùng đơn hàng TC_CD_01</t>
-  </si>
-  <si>
     <t>B. VALIDATION TRƯỚC KHI TẠO ĐƠN</t>
   </si>
   <si>
-    <t>CD_02</t>
-  </si>
-  <si>
     <t>Ràng buộc sản phẩm</t>
   </si>
   <si>
-    <t>TC_CD_03</t>
-  </si>
-  <si>
     <t>Negative</t>
   </si>
   <si>
@@ -135,31 +116,19 @@
     <t>Hệ thống KHÔNG thực hiện lệnh tạo đơn. Hiển thị thông báo lỗi: "Bạn phải chọn sản phẩm".</t>
   </si>
   <si>
-    <t>TC_CD_04</t>
-  </si>
-  <si>
     <t>Chặn tạo đơn khi sản phẩm IMEI chưa chọn mã (SL=0)</t>
   </si>
   <si>
     <t>Hệ thống chặn lệnh. Hiển thị thông báo lỗi: "Số lượng sản phẩm phải lớn hơn 0".</t>
   </si>
   <si>
-    <t>TC_CD_05</t>
-  </si>
-  <si>
     <t>Chặn tạo đơn khi sản phẩm Lô-HSD chưa chọn lô (SL=0)</t>
   </si>
   <si>
     <t>C. CẬP NHẬT TỒN KHO SAU KHI TẠO ĐƠN</t>
   </si>
   <si>
-    <t>CD_03</t>
-  </si>
-  <si>
     <t>Cập nhật tồn kho</t>
-  </si>
-  <si>
-    <t>TC_CD_06</t>
   </si>
   <si>
     <t>Kiểm tra trừ tồn kho sản phẩm Thường sau khi tạo đơn</t>
@@ -179,33 +148,15 @@
     <t>Tồn kho sản phẩm giảm xuống còn 4.</t>
   </si>
   <si>
-    <t>TC_CD_07</t>
-  </si>
-  <si>
     <t>Kiểm tra trừ tồn kho sản phẩm IMEI</t>
   </si>
   <si>
-    <t>TC_CD_08</t>
-  </si>
-  <si>
     <t>Kiểm tra trừ tồn kho sản phẩm Lô-HSD</t>
   </si>
   <si>
-    <t>TC_CD_09</t>
-  </si>
-  <si>
     <t>Medium</t>
   </si>
   <si>
-    <t>CD_04</t>
-  </si>
-  <si>
-    <t>TC_CD_10</t>
-  </si>
-  <si>
-    <t>TC_CD_11</t>
-  </si>
-  <si>
     <t>Tạo đơn KH phải trả = 143.000đ</t>
   </si>
   <si>
@@ -215,9 +166,6 @@
     <t>Tổng doanh thu tăng thêm 143.000đ. Đơn hàng xuất hiện trong báo cáo với giá trị đúng.</t>
   </si>
   <si>
-    <t>CD_05</t>
-  </si>
-  <si>
     <t>Xử lý đồng thời</t>
   </si>
   <si>
@@ -225,9 +173,6 @@
   </si>
   <si>
     <t>Hệ thống chỉ tạo 1 đơn duy nhất (không tạo 3 đơn trùng). Tồn kho giảm 1 lần (10 → 9), không giảm 3 lần.</t>
-  </si>
-  <si>
-    <t>CD_06</t>
   </si>
   <si>
     <t>Ngoại lệ kết nối</t>
@@ -332,6 +277,60 @@
   <si>
     <t xml:space="preserve">Hệ thống hiển thị thông báo lỗi "Đơn hàng đã được lưu tạm. Và sẽ tự động gửi khi có mạng"
 </t>
+  </si>
+  <si>
+    <t>CO_TC_05</t>
+  </si>
+  <si>
+    <t>CO_TC_01</t>
+  </si>
+  <si>
+    <t>CO_TC_02</t>
+  </si>
+  <si>
+    <t>Cùng đơn hàng CO_TC_01</t>
+  </si>
+  <si>
+    <t>CO_TC_03</t>
+  </si>
+  <si>
+    <t>CO_TC_04</t>
+  </si>
+  <si>
+    <t>CO_TC_06</t>
+  </si>
+  <si>
+    <t>CO_TC_07</t>
+  </si>
+  <si>
+    <t>CO_TC_08</t>
+  </si>
+  <si>
+    <t>CO_TC_09</t>
+  </si>
+  <si>
+    <t>CO_TC_10</t>
+  </si>
+  <si>
+    <t>CO_TC_11</t>
+  </si>
+  <si>
+    <t>CO_01</t>
+  </si>
+  <si>
+    <t>CO_02</t>
+  </si>
+  <si>
+    <t>CO_03</t>
+  </si>
+  <si>
+    <t>CO_04</t>
+  </si>
+  <si>
+    <t>CO_05</t>
+  </si>
+  <si>
+    <t>CO_06</t>
   </si>
 </sst>
 </file>
@@ -808,71 +807,71 @@
     </row>
     <row r="3" spans="1:11" ht="70.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="C3" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="E3" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="F3" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="G3" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="H3" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="I3" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="H3" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>20</v>
-      </c>
       <c r="J3" s="2" t="s">
-        <v>72</v>
+        <v>54</v>
       </c>
       <c r="K3" s="2"/>
     </row>
     <row r="4" spans="1:11" ht="55.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>12</v>
+        <v>90</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H4" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D4" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>24</v>
-      </c>
       <c r="I4" s="2" t="s">
-        <v>25</v>
+        <v>81</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>72</v>
+        <v>54</v>
       </c>
       <c r="K4" s="2"/>
     </row>
     <row r="5" spans="1:11" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B5" s="7"/>
       <c r="C5" s="7"/>
@@ -887,102 +886,102 @@
     </row>
     <row r="6" spans="1:11" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="H6" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="I6" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="J6" s="2" t="s">
         <v>29</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="I6" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="J6" s="2" t="s">
-        <v>35</v>
       </c>
       <c r="K6" s="2"/>
     </row>
     <row r="7" spans="1:11" ht="59.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>27</v>
+        <v>91</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" s="2" t="s">
-        <v>36</v>
+        <v>83</v>
       </c>
       <c r="D7" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="E7" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>37</v>
-      </c>
       <c r="G7" s="2" t="s">
-        <v>75</v>
+        <v>57</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>76</v>
+        <v>58</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="K7" s="2"/>
     </row>
     <row r="8" spans="1:11" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>27</v>
+        <v>91</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" s="2" t="s">
-        <v>39</v>
+        <v>78</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>77</v>
+        <v>59</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>89</v>
+        <v>71</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>79</v>
+        <v>61</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="K8" s="2"/>
     </row>
     <row r="9" spans="1:11" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="6" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
@@ -997,102 +996,102 @@
     </row>
     <row r="10" spans="1:11" ht="64.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>42</v>
+        <v>92</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>43</v>
+        <v>34</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>44</v>
+        <v>84</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="K10" s="2"/>
     </row>
     <row r="11" spans="1:11" ht="78" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>42</v>
+        <v>92</v>
       </c>
       <c r="B11" s="2"/>
       <c r="C11" s="2" t="s">
-        <v>50</v>
+        <v>85</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>51</v>
+        <v>40</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>73</v>
+        <v>55</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>81</v>
+        <v>63</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>74</v>
+        <v>56</v>
       </c>
       <c r="K11" s="2"/>
     </row>
     <row r="12" spans="1:11" ht="64.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>42</v>
+        <v>92</v>
       </c>
       <c r="B12" s="2"/>
       <c r="C12" s="2" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>78</v>
+        <v>60</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>91</v>
+        <v>73</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>80</v>
+        <v>62</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="K12" s="2"/>
     </row>
     <row r="13" spans="1:11" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="6" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="B13" s="7"/>
       <c r="C13" s="7"/>
@@ -1107,38 +1106,38 @@
     </row>
     <row r="14" spans="1:11" ht="61.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>56</v>
+        <v>93</v>
       </c>
       <c r="B14" s="2"/>
       <c r="C14" s="2" t="s">
-        <v>54</v>
+        <v>87</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>55</v>
+        <v>42</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>87</v>
+        <v>69</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>59</v>
+        <v>43</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>92</v>
+        <v>74</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>60</v>
+        <v>44</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>61</v>
+        <v>45</v>
       </c>
       <c r="K14" s="2"/>
     </row>
     <row r="15" spans="1:11" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="6" t="s">
-        <v>71</v>
+        <v>53</v>
       </c>
       <c r="B15" s="7"/>
       <c r="C15" s="7"/>
@@ -1153,40 +1152,40 @@
     </row>
     <row r="16" spans="1:11" ht="64.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
-        <v>62</v>
+        <v>94</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>63</v>
+        <v>46</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>57</v>
+        <v>88</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>64</v>
+        <v>47</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>93</v>
+        <v>75</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>84</v>
+        <v>66</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>65</v>
+        <v>48</v>
       </c>
       <c r="K16" s="2"/>
     </row>
     <row r="17" spans="1:11" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="6" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="B17" s="7"/>
       <c r="C17" s="7"/>
@@ -1201,45 +1200,45 @@
     </row>
     <row r="18" spans="1:11" ht="70.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
-        <v>66</v>
+        <v>95</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>58</v>
+        <v>89</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>69</v>
+        <v>51</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>94</v>
+        <v>76</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>70</v>
+        <v>52</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>95</v>
+        <v>77</v>
       </c>
       <c r="K18" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="A2:K2"/>
     <mergeCell ref="A5:K5"/>
     <mergeCell ref="A15:K15"/>
     <mergeCell ref="A13:K13"/>
     <mergeCell ref="A17:K17"/>
     <mergeCell ref="A9:K9"/>
-    <mergeCell ref="A2:K2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>